<commit_message>
Changes to the ME system and others. Draws from other files.
</commit_message>
<xml_diff>
--- a/bull_comparison.xlsx
+++ b/bull_comparison.xlsx
@@ -5,12 +5,12 @@
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arvel\OneDrive\Desktop\Other\EPDs\2026EPD\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\arvel\OneDrive\Desktop\Other\EPDs\DHOLL_EPDS\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E0649F22-F37D-46E7-A5FE-652AE0E38DB5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0DE82E8E-6186-468D-A130-EB621B82DBDF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="1650" yWindow="2235" windowWidth="21600" windowHeight="11340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="5835" yWindow="2190" windowWidth="21600" windowHeight="11340" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet0" sheetId="1" r:id="rId1"/>
@@ -564,7 +564,8 @@
     <col min="15" max="16" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="17" max="17" width="4.7109375" bestFit="1" customWidth="1"/>
     <col min="18" max="18" width="3.7109375" bestFit="1" customWidth="1"/>
-    <col min="19" max="20" width="5" bestFit="1" customWidth="1"/>
+    <col min="19" max="19" width="5" bestFit="1" customWidth="1"/>
+    <col min="20" max="20" width="5" customWidth="1"/>
     <col min="21" max="21" width="5.140625" bestFit="1" customWidth="1"/>
     <col min="22" max="22" width="5.7109375" bestFit="1" customWidth="1"/>
     <col min="23" max="23" width="5.85546875" bestFit="1" customWidth="1"/>

</xml_diff>